<commit_message>
Add three holographic tape roll samples to radium stock sheet
Quantities left blank to be filled in later.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3syLEqJFFyzLQTDmCuMjz
</commit_message>
<xml_diff>
--- a/Radium_Samples_Stock.xlsx
+++ b/Radium_Samples_Stock.xlsx
@@ -33,7 +33,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +43,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -72,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -81,6 +86,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -728,6 +739,81 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1085850" cy="1143000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1009650" cy="1143000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="971550" cy="1143000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1030,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1746,25 +1832,94 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="C26" s="4" t="inlineStr">
+    <row r="25" ht="95" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pink sequin-dot holographic tape roll</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="5" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Photo 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="95" customHeight="1">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Gold sequin-dot holographic tape roll</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="5" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Photo 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="95" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Silver sequin-dot holographic tape roll</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="5" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Photo 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Total (Meters)</t>
         </is>
       </c>
-      <c r="D26" s="5">
-        <f>SUMIF(E2:E24,"Meters",D2:D24)</f>
+      <c r="D29" s="7">
+        <f>SUMIF(E2:E27,"Meters",D2:D27)</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="C27" s="4" t="inlineStr">
+    <row r="30">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Total (Yards)</t>
         </is>
       </c>
-      <c r="D27" s="5">
-        <f>SUMIF(E2:E24,"Yards",D2:D24)</f>
+      <c r="D30" s="7">
+        <f>SUMIF(E2:E27,"Yards",D2:D27)</f>
         <v/>
       </c>
     </row>

</xml_diff>